<commit_message>
[Feat] Add Group ID
</commit_message>
<xml_diff>
--- a/Assets/Excel/DialogueTable.xlsx
+++ b/Assets/Excel/DialogueTable.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kjghk\OneDrive\Desktop\mindsneakers\Assets\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85647133-2800-427C-81AC-974A8CEAAADC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{892FBBD8-9835-4040-984E-56E51116C72A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DoubleDialogue" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="25">
   <si>
     <t>Hero_Normal</t>
   </si>
@@ -94,6 +94,18 @@
   </si>
   <si>
     <t>Image</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Text4</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Text5</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Text6</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -549,7 +561,7 @@
         <v>9</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -575,7 +587,7 @@
         <v>12</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -601,7 +613,7 @@
         <v>9</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[Feat] Add Scene Change
</commit_message>
<xml_diff>
--- a/Assets/Excel/DialogueTable.xlsx
+++ b/Assets/Excel/DialogueTable.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kjghk\OneDrive\Desktop\mindsneakers\Assets\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB5AC9E5-FAE7-49E6-AC2A-CDEFE0EBC83E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A602356D-5300-4320-B87E-41275C6E2FBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1958,7 +1958,7 @@
     </row>
     <row r="2" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B2">
         <v>1001</v>
@@ -1984,7 +1984,7 @@
     </row>
     <row r="3" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B3">
         <v>1002</v>
@@ -2010,7 +2010,7 @@
     </row>
     <row r="4" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B4">
         <v>1003</v>
@@ -2036,7 +2036,7 @@
     </row>
     <row r="5" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B5">
         <v>1004</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="6" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B6">
         <v>1005</v>
@@ -2088,7 +2088,7 @@
     </row>
     <row r="7" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B7">
         <v>1006</v>
@@ -2114,7 +2114,7 @@
     </row>
     <row r="8" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B8">
         <v>1007</v>
@@ -2140,7 +2140,7 @@
     </row>
     <row r="9" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B9">
         <v>1008</v>
@@ -2166,7 +2166,7 @@
     </row>
     <row r="10" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B10">
         <v>1009</v>
@@ -2192,7 +2192,7 @@
     </row>
     <row r="11" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B11">
         <v>1010</v>
@@ -2218,7 +2218,7 @@
     </row>
     <row r="12" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B12">
         <v>1011</v>
@@ -2244,7 +2244,7 @@
     </row>
     <row r="13" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B13">
         <v>1012</v>
@@ -2270,7 +2270,7 @@
     </row>
     <row r="14" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A14">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B14">
         <v>1013</v>
@@ -2296,7 +2296,7 @@
     </row>
     <row r="15" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B15">
         <v>1014</v>
@@ -2322,7 +2322,7 @@
     </row>
     <row r="16" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B16">
         <v>1015</v>
@@ -2348,7 +2348,7 @@
     </row>
     <row r="17" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B17">
         <v>1016</v>
@@ -2374,7 +2374,7 @@
     </row>
     <row r="18" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B18">
         <v>1017</v>
@@ -2400,7 +2400,7 @@
     </row>
     <row r="19" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B19">
         <v>1018</v>
@@ -2426,7 +2426,7 @@
     </row>
     <row r="20" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B20">
         <v>1019</v>
@@ -2452,7 +2452,7 @@
     </row>
     <row r="21" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B21">
         <v>1020</v>
@@ -2478,7 +2478,7 @@
     </row>
     <row r="22" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B22">
         <v>1021</v>
@@ -2504,7 +2504,7 @@
     </row>
     <row r="23" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A23">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B23">
         <v>1022</v>
@@ -2530,7 +2530,7 @@
     </row>
     <row r="24" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B24">
         <v>1023</v>
@@ -2556,7 +2556,7 @@
     </row>
     <row r="25" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B25">
         <v>1024</v>
@@ -2582,7 +2582,7 @@
     </row>
     <row r="26" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B26">
         <v>1025</v>
@@ -2608,7 +2608,7 @@
     </row>
     <row r="27" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A27">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B27">
         <v>1026</v>
@@ -2634,7 +2634,7 @@
     </row>
     <row r="28" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B28">
         <v>1027</v>
@@ -2660,7 +2660,7 @@
     </row>
     <row r="29" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B29">
         <v>1028</v>
@@ -2686,7 +2686,7 @@
     </row>
     <row r="30" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B30">
         <v>1029</v>
@@ -2712,7 +2712,7 @@
     </row>
     <row r="31" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B31">
         <v>1030</v>
@@ -2738,7 +2738,7 @@
     </row>
     <row r="32" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B32">
         <v>1031</v>
@@ -2764,7 +2764,7 @@
     </row>
     <row r="33" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B33">
         <v>1032</v>
@@ -2790,7 +2790,7 @@
     </row>
     <row r="34" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B34">
         <v>1033</v>
@@ -2816,7 +2816,7 @@
     </row>
     <row r="35" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B35">
         <v>1034</v>
@@ -2842,7 +2842,7 @@
     </row>
     <row r="36" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B36">
         <v>1035</v>
@@ -2868,7 +2868,7 @@
     </row>
     <row r="37" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B37">
         <v>1036</v>
@@ -2894,7 +2894,7 @@
     </row>
     <row r="38" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B38">
         <v>1037</v>
@@ -2920,7 +2920,7 @@
     </row>
     <row r="39" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A39">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B39">
         <v>1038</v>
@@ -2946,7 +2946,7 @@
     </row>
     <row r="40" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B40">
         <v>1039</v>

</xml_diff>